<commit_message>
Fixed the links to other files
</commit_message>
<xml_diff>
--- a/AMD.xlsx
+++ b/AMD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/Stocks/Data/Stocks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE85E417-1D62-A04C-B29D-EC646EF7EB6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9B665F-1F69-C147-8FD4-2B704A7A0AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -1176,20 +1176,19 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Sheet1"/>
+      <sheetName val="1. List_AutomaticData"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0">
         <row r="3">
           <cell r="C3">
-            <v>205.37</v>
+            <v>278.39</v>
           </cell>
         </row>
       </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1617,7 +1616,7 @@
       </c>
       <c r="C3" s="38">
         <f>[1]Sheet1!$C$3</f>
-        <v>205.37</v>
+        <v>278.39</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.2">
@@ -1637,7 +1636,7 @@
       </c>
       <c r="C9" s="94">
         <f>C3*'Statement Q'!J138</f>
-        <v>334753.10000000003</v>
+        <v>453775.69999999995</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.2">

</xml_diff>